<commit_message>
feat: break tracking, SQLite backend, webhook notifications
- Break tracking: pause -r REASON logs break info to column L
- SQLite backend: db.py, enabled via WORKLOG_DB=sqlite
- Webhook notifications: webhook.py, enabled via WORKLOG_WEBHOOK_URL
- build.py: added col L, shifted hidden helpers M-R
- auto.py: init SQLite on startup
- how_to_use.md & README.md: updated docs
</commit_message>
<xml_diff>
--- a/worklog.xlsx
+++ b/worklog.xlsx
@@ -18065,10 +18065,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
-      <c r="H2" s="25" t="n"/>
+      <c r="H2" s="35" t="n">
+        <v>46224</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18141,8 +18143,36 @@
       </c>
     </row>
     <row r="5">
-      <c r="D5" s="25" t="n"/>
-      <c r="F5" s="28" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KPI-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Fix the test case MagicBean</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="n">
+        <v>46224</v>
+      </c>
+      <c r="E5" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="28">
+        <f>IF(E5&lt;&gt;"",E5*7.5,"")</f>
+        <v/>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
       <c r="H5" s="25" t="n"/>
     </row>
     <row r="6">

</xml_diff>